<commit_message>
Revision after external review: Cross & Vesely reading and launch variants by starting knowledge, K_need infeasible case, admissibility screen first (Table 6, Fig. 8), hard exposure limit, tuned threshold baseline and ablations, replicated and closed-loop estimation
</commit_message>
<xml_diff>
--- a/supplementary/KMC_Worksheet.xlsx
+++ b/supplementary/KMC_Worksheet.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
   <authors>
     <author>Unknown Author</author>
   </authors>
@@ -40,6 +40,27 @@
           <t xml:space="preserve">Override column: Org X rounds the calibrated values to the card of S1, Sec. 3.5. Clear a cell to use the calibrated value.</t>
         </r>
       </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>0</xdr:col>
+                <xdr:colOff>79</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>5</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>31</xdr:colOff>
+                <xdr:row>4</xdr:row>
+                <xdr:rowOff>19</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
     </comment>
   </commentList>
 </comments>
@@ -492,7 +513,7 @@
     <t xml:space="preserve">R6</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 3: M &lt; M_req, K ≥ K_need and hazard ≤ h_max → integrated test.  Step 4 (and 3b): otherwise the activity with the largest net K rate = K gain − hazard·δ_K.  Always screen the activity against cost, schedule and exposure (step 6) and re-assess after every result.</t>
+    <t xml:space="preserve">Step 0 first: screen every candidate activity against cost, schedule and exposure and keep only the admissible ones.  Step 3: M &lt; M_req, K ≥ K_need and hazard ≤ h_max → integrated test.  Step 4 (and 3b): otherwise the admissible activity with the largest net K rate = K gain − hazard·δ_K.  Re-assess after every result.</t>
   </si>
 </sst>
 </file>

</xml_diff>